<commit_message>
Regenerate all workbooks with the Industry column
Rebuild every Industry-bearing book from current data so the tracked
snapshots carry the new Industry column beside Sector (24 books):
country-archetype family (book/otc/52w-high/midcap/cheap8/ret12m-neg/pb-sub1),
inflection family, top-by-archetype, truly-XR, forensic-XR, segment-detail,
NMS book + candidates, harvard, country workbook, and top_n_by_country
(+ inflection/otc/52w-high). Companion CSVs regenerated in the same runs.

Verified Industry present and aligned (e.g. pb_sub1/book/segment/truly-XR
Sector@5 Industry@6; nms Global_Top_100 Sector@6 Industry@7).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -10865,7 +10865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -10874,12 +10874,13 @@
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="4" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="4" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -10899,6 +10900,7 @@
       <c r="J1" s="10" t="n"/>
       <c r="K1" s="10" t="n"/>
       <c r="L1" s="10" t="n"/>
+      <c r="M1" s="10" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="13" t="inlineStr">
@@ -10926,27 +10928,32 @@
           <t>Sector</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="I3" s="15" t="inlineStr">
+      <c r="J3" s="15" t="inlineStr">
         <is>
           <t>P/B</t>
         </is>
       </c>
-      <c r="J3" s="15" t="inlineStr">
+      <c r="K3" s="15" t="inlineStr">
         <is>
           <t>Div %</t>
         </is>
       </c>
-      <c r="K3" s="15" t="inlineStr">
+      <c r="L3" s="15" t="inlineStr">
         <is>
           <t>P/S</t>
         </is>
@@ -10976,21 +10983,24 @@
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="G4" s="21" t="inlineStr">
+      <c r="G4" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H4" s="22" t="n">
+      <c r="I4" s="22" t="n">
         <v>1.337323840582209</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="J4" s="22" t="n">
         <v>0.2358961702739243</v>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="K4" s="23" t="n">
         <v>2.42</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="L4" s="22" t="n">
         <v>0.19885361</v>
       </c>
     </row>
@@ -11018,21 +11028,26 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G5" s="24" t="inlineStr">
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Internet &amp; Direct Marketing Retail</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="I5" s="22" t="n">
         <v>1.2546601832671</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="J5" s="22" t="n">
         <v>0.3895122570757942</v>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="K5" s="23" t="n">
         <v>2.0299999</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="L5" s="22" t="n">
         <v>0.33442965</v>
       </c>
     </row>
@@ -11060,21 +11075,26 @@
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="G6" s="21" t="inlineStr">
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="I6" s="22" t="n">
         <v>1.224320047113935</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="J6" s="22" t="n">
         <v>0.5975976</v>
       </c>
-      <c r="J6" s="23" t="n">
+      <c r="K6" s="23" t="n">
         <v>6.79</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="L6" s="22" t="n">
         <v>0.6178304</v>
       </c>
     </row>
@@ -11102,23 +11122,28 @@
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Interactive Media &amp; Services</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="I7" s="22" t="n">
         <v>1.213706119342358</v>
       </c>
-      <c r="I7" s="22" t="n">
+      <c r="J7" s="22" t="n">
         <v>0.64855975</v>
       </c>
-      <c r="J7" s="25" t="inlineStr">
+      <c r="K7" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K7" s="22" t="n">
+      <c r="L7" s="22" t="n">
         <v>1.076399494270387</v>
       </c>
     </row>
@@ -11146,21 +11171,26 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="I8" s="22" t="n">
         <v>1.201964122014842</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="J8" s="22" t="n">
         <v>0.63487464</v>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="K8" s="23" t="n">
         <v>2.4300002</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="L8" s="22" t="n">
         <v>0.30129302</v>
       </c>
     </row>
@@ -11188,21 +11218,26 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="G9" s="21" t="inlineStr">
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Oil, Gas &amp; Consumable Fuels</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="I9" s="22" t="n">
         <v>1.196379645329934</v>
       </c>
-      <c r="I9" s="22" t="n">
+      <c r="J9" s="22" t="n">
         <v>0.3814184820374598</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="K9" s="23" t="n">
         <v>2.77</v>
       </c>
-      <c r="K9" s="22" t="n">
+      <c r="L9" s="22" t="n">
         <v>0.47579452</v>
       </c>
     </row>
@@ -11230,21 +11265,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G10" s="21" t="inlineStr">
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Electrical Equipment</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="I10" s="22" t="n">
         <v>1.19387677304337</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="J10" s="22" t="n">
         <v>0.4305136</v>
       </c>
-      <c r="J10" s="23" t="n">
+      <c r="K10" s="23" t="n">
         <v>3.28</v>
       </c>
-      <c r="K10" s="22" t="n">
+      <c r="L10" s="22" t="n">
         <v>0.3348663</v>
       </c>
     </row>
@@ -11272,21 +11312,26 @@
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="I11" s="22" t="n">
         <v>1.187594330021412</v>
       </c>
-      <c r="I11" s="22" t="n">
+      <c r="J11" s="22" t="n">
         <v>0.82867485</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="K11" s="23" t="n">
         <v>3.55</v>
       </c>
-      <c r="K11" s="22" t="n">
+      <c r="L11" s="22" t="n">
         <v>0.45901608</v>
       </c>
     </row>
@@ -11314,21 +11359,26 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Auto Components</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="I12" s="22" t="n">
         <v>1.172504383176419</v>
       </c>
-      <c r="I12" s="22" t="n">
+      <c r="J12" s="22" t="n">
         <v>0.605814</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="K12" s="23" t="n">
         <v>4.21</v>
       </c>
-      <c r="K12" s="22" t="n">
+      <c r="L12" s="22" t="n">
         <v>0.5752</v>
       </c>
     </row>
@@ -11356,21 +11406,24 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G13" s="21" t="inlineStr">
+      <c r="G13" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H13" s="22" t="n">
+      <c r="I13" s="22" t="n">
         <v>1.17208086301225</v>
       </c>
-      <c r="I13" s="22" t="n">
+      <c r="J13" s="22" t="n">
         <v>0.3329555299332747</v>
       </c>
-      <c r="J13" s="23" t="n">
+      <c r="K13" s="23" t="n">
         <v>2.21</v>
       </c>
-      <c r="K13" s="22" t="n">
+      <c r="L13" s="22" t="n">
         <v>0.13220902</v>
       </c>
     </row>
@@ -11398,21 +11451,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H14" s="22" t="n">
+      <c r="I14" s="22" t="n">
         <v>1.168783020601786</v>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="J14" s="22" t="n">
         <v>0.6870092</v>
       </c>
-      <c r="J14" s="23" t="n">
+      <c r="K14" s="23" t="n">
         <v>2.53</v>
       </c>
-      <c r="K14" s="22" t="n">
+      <c r="L14" s="22" t="n">
         <v>0.9294438</v>
       </c>
     </row>
@@ -11440,21 +11498,26 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G15" s="21" t="inlineStr">
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Distributors</t>
+        </is>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H15" s="22" t="n">
+      <c r="I15" s="22" t="n">
         <v>1.164103836676694</v>
       </c>
-      <c r="I15" s="22" t="n">
+      <c r="J15" s="22" t="n">
         <v>0.5009125</v>
       </c>
-      <c r="J15" s="23" t="n">
+      <c r="K15" s="23" t="n">
         <v>8.33</v>
       </c>
-      <c r="K15" s="22" t="n">
+      <c r="L15" s="22" t="n">
         <v>1.6125863</v>
       </c>
     </row>
@@ -11482,21 +11545,24 @@
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="G16" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H16" s="22" t="n">
+      <c r="I16" s="22" t="n">
         <v>1.163897066936411</v>
       </c>
-      <c r="I16" s="22" t="n">
+      <c r="J16" s="22" t="n">
         <v>0.9925171574056828</v>
       </c>
-      <c r="J16" s="23" t="n">
+      <c r="K16" s="23" t="n">
         <v>4.9200002</v>
       </c>
-      <c r="K16" s="22" t="n">
+      <c r="L16" s="22" t="n">
         <v>1.2269952</v>
       </c>
     </row>
@@ -11524,23 +11590,26 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="G17" s="21" t="inlineStr">
+      <c r="G17" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H17" s="22" t="n">
+      <c r="I17" s="22" t="n">
         <v>1.152290474548095</v>
       </c>
-      <c r="I17" s="22" t="n">
+      <c r="J17" s="22" t="n">
         <v>0.5449940720767228</v>
       </c>
-      <c r="J17" s="25" t="inlineStr">
+      <c r="K17" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K17" s="22" t="n">
+      <c r="L17" s="22" t="n">
         <v>0.8796080168298662</v>
       </c>
     </row>
@@ -11568,21 +11637,24 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G18" s="21" t="inlineStr">
+      <c r="G18" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H18" s="22" t="n">
+      <c r="I18" s="22" t="n">
         <v>1.151619597547656</v>
       </c>
-      <c r="I18" s="22" t="n">
+      <c r="J18" s="22" t="n">
         <v>0.3869141557375681</v>
       </c>
-      <c r="J18" s="23" t="n">
+      <c r="K18" s="23" t="n">
         <v>2.79</v>
       </c>
-      <c r="K18" s="22" t="n">
+      <c r="L18" s="22" t="n">
         <v>0.3518272690665361</v>
       </c>
     </row>
@@ -11610,23 +11682,28 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="G19" s="24" t="inlineStr">
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H19" s="22" t="n">
+      <c r="I19" s="22" t="n">
         <v>1.145311286187199</v>
       </c>
-      <c r="I19" s="22" t="n">
+      <c r="J19" s="22" t="n">
         <v>0.07192945000000001</v>
       </c>
-      <c r="J19" s="25" t="inlineStr">
+      <c r="K19" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K19" s="22" t="n">
+      <c r="L19" s="22" t="n">
         <v>3.837890044653707</v>
       </c>
     </row>
@@ -11654,21 +11731,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr">
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+      <c r="H20" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H20" s="22" t="n">
+      <c r="I20" s="22" t="n">
         <v>1.129692505982211</v>
       </c>
-      <c r="I20" s="22" t="n">
+      <c r="J20" s="22" t="n">
         <v>0.3569352</v>
       </c>
-      <c r="J20" s="23" t="n">
+      <c r="K20" s="23" t="n">
         <v>2.02</v>
       </c>
-      <c r="K20" s="22" t="n">
+      <c r="L20" s="22" t="n">
         <v>0.4588686</v>
       </c>
     </row>
@@ -11696,21 +11778,24 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G21" s="19" t="inlineStr">
+      <c r="G21" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>YELLOW</t>
         </is>
       </c>
-      <c r="H21" s="22" t="n">
+      <c r="I21" s="22" t="n">
         <v>1.128749512459602</v>
       </c>
-      <c r="I21" s="22" t="n">
+      <c r="J21" s="22" t="n">
         <v>0.3574623360623071</v>
       </c>
-      <c r="J21" s="23" t="n">
+      <c r="K21" s="23" t="n">
         <v>2.0299999</v>
       </c>
-      <c r="K21" s="22" t="n">
+      <c r="L21" s="22" t="n">
         <v>0.20222703</v>
       </c>
     </row>
@@ -11738,23 +11823,26 @@
           <t>Health Care</t>
         </is>
       </c>
-      <c r="G22" s="24" t="inlineStr">
+      <c r="G22" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H22" s="22" t="n">
+      <c r="I22" s="22" t="n">
         <v>1.126098255566523</v>
       </c>
-      <c r="I22" s="22" t="n">
+      <c r="J22" s="22" t="n">
         <v>0.4404573070670534</v>
       </c>
-      <c r="J22" s="25" t="inlineStr">
+      <c r="K22" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K22" s="22" t="n">
+      <c r="L22" s="22" t="n">
         <v>1.1023238</v>
       </c>
     </row>
@@ -11782,23 +11870,28 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G23" s="24" t="inlineStr">
+      <c r="G23" s="20" t="inlineStr">
+        <is>
+          <t>IT Services</t>
+        </is>
+      </c>
+      <c r="H23" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H23" s="22" t="n">
+      <c r="I23" s="22" t="n">
         <v>1.114077191724072</v>
       </c>
-      <c r="I23" s="22" t="n">
+      <c r="J23" s="22" t="n">
         <v>0.14073937</v>
       </c>
-      <c r="J23" s="25" t="inlineStr">
+      <c r="K23" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K23" s="22" t="n">
+      <c r="L23" s="22" t="n">
         <v>0.2087546874822286</v>
       </c>
     </row>
@@ -11826,23 +11919,28 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G24" s="24" t="inlineStr">
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>Internet &amp; Direct Marketing Retail</t>
+        </is>
+      </c>
+      <c r="H24" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H24" s="22" t="n">
+      <c r="I24" s="22" t="n">
         <v>1.101049539651115</v>
       </c>
-      <c r="I24" s="22" t="n">
+      <c r="J24" s="22" t="n">
         <v>0.2626032</v>
       </c>
-      <c r="J24" s="25" t="inlineStr">
+      <c r="K24" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K24" s="22" t="n">
+      <c r="L24" s="22" t="n">
         <v>1.151275859708347</v>
       </c>
     </row>
@@ -11870,21 +11968,26 @@
           <t>Health Care</t>
         </is>
       </c>
-      <c r="G25" s="24" t="inlineStr">
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H25" s="22" t="n">
+      <c r="I25" s="22" t="n">
         <v>1.09772165902702</v>
       </c>
-      <c r="I25" s="22" t="n">
+      <c r="J25" s="22" t="n">
         <v>0.37324485</v>
       </c>
-      <c r="J25" s="23" t="n">
+      <c r="K25" s="23" t="n">
         <v>6.3</v>
       </c>
-      <c r="K25" s="22" t="n">
+      <c r="L25" s="22" t="n">
         <v>1.126572896664314</v>
       </c>
     </row>
@@ -11912,23 +12015,26 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G26" s="21" t="inlineStr">
+      <c r="G26" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H26" s="22" t="n">
+      <c r="I26" s="22" t="n">
         <v>1.09623561521307</v>
       </c>
-      <c r="I26" s="22" t="n">
+      <c r="J26" s="22" t="n">
         <v>1.168593365730836</v>
       </c>
-      <c r="J26" s="25" t="inlineStr">
+      <c r="K26" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K26" s="22" t="n">
+      <c r="L26" s="22" t="n">
         <v>1.8895935</v>
       </c>
     </row>
@@ -11956,21 +12062,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G27" s="21" t="inlineStr">
+      <c r="G27" s="20" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H27" s="22" t="n">
+      <c r="I27" s="22" t="n">
         <v>1.095490665810664</v>
       </c>
-      <c r="I27" s="22" t="n">
+      <c r="J27" s="22" t="n">
         <v>0.2918288</v>
       </c>
-      <c r="J27" s="23" t="n">
+      <c r="K27" s="23" t="n">
         <v>7.0700005</v>
       </c>
-      <c r="K27" s="22" t="n">
+      <c r="L27" s="22" t="n">
         <v>0.38369063</v>
       </c>
     </row>
@@ -11998,21 +12109,24 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G28" s="21" t="inlineStr">
+      <c r="G28" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H28" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H28" s="22" t="n">
+      <c r="I28" s="22" t="n">
         <v>1.082675977629569</v>
       </c>
-      <c r="I28" s="22" t="n">
+      <c r="J28" s="22" t="n">
         <v>1.0374141</v>
       </c>
-      <c r="J28" s="23" t="n">
+      <c r="K28" s="23" t="n">
         <v>0.5599999999999999</v>
       </c>
-      <c r="K28" s="22" t="n">
+      <c r="L28" s="22" t="n">
         <v>2.9770486</v>
       </c>
     </row>
@@ -12040,23 +12154,28 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G29" s="21" t="inlineStr">
+      <c r="G29" s="20" t="inlineStr">
+        <is>
+          <t>Electronic Equipment, Instruments &amp; Components</t>
+        </is>
+      </c>
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H29" s="22" t="n">
+      <c r="I29" s="22" t="n">
         <v>1.081940931362408</v>
       </c>
-      <c r="I29" s="22" t="n">
+      <c r="J29" s="22" t="n">
         <v>0.5689394</v>
       </c>
-      <c r="J29" s="25" t="inlineStr">
+      <c r="K29" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K29" s="22" t="n">
+      <c r="L29" s="22" t="n">
         <v>0.9480809</v>
       </c>
     </row>
@@ -12084,21 +12203,26 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="G30" s="24" t="inlineStr">
+      <c r="G30" s="20" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="H30" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H30" s="22" t="n">
+      <c r="I30" s="22" t="n">
         <v>1.081044056088647</v>
       </c>
-      <c r="I30" s="22" t="n">
+      <c r="J30" s="22" t="n">
         <v>0.36005497</v>
       </c>
-      <c r="J30" s="23" t="n">
+      <c r="K30" s="23" t="n">
         <v>3.52</v>
       </c>
-      <c r="K30" s="22" t="n">
+      <c r="L30" s="22" t="n">
         <v>0.26927328</v>
       </c>
     </row>
@@ -12126,23 +12250,26 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G31" s="24" t="inlineStr">
+      <c r="G31" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H31" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H31" s="22" t="n">
+      <c r="I31" s="22" t="n">
         <v>1.077025085586687</v>
       </c>
-      <c r="I31" s="22" t="n">
+      <c r="J31" s="22" t="n">
         <v>0.6557044396837195</v>
       </c>
-      <c r="J31" s="25" t="inlineStr">
+      <c r="K31" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K31" s="22" t="n">
+      <c r="L31" s="22" t="n">
         <v>0.7902293526088751</v>
       </c>
     </row>
@@ -12170,21 +12297,24 @@
           <t>Health Care</t>
         </is>
       </c>
-      <c r="G32" s="24" t="inlineStr">
+      <c r="G32" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H32" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H32" s="22" t="n">
+      <c r="I32" s="22" t="n">
         <v>1.076618108296869</v>
       </c>
-      <c r="I32" s="22" t="n">
+      <c r="J32" s="22" t="n">
         <v>0.4577384913211642</v>
       </c>
-      <c r="J32" s="23" t="n">
+      <c r="K32" s="23" t="n">
         <v>5.71</v>
       </c>
-      <c r="K32" s="22" t="n">
+      <c r="L32" s="22" t="n">
         <v>0.5612516400000001</v>
       </c>
     </row>
@@ -12210,21 +12340,24 @@
       <c r="F33" s="20" t="n">
         <v/>
       </c>
-      <c r="G33" s="21" t="inlineStr">
+      <c r="G33" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H33" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H33" s="22" t="n">
+      <c r="I33" s="22" t="n">
         <v>1.072794052555671</v>
       </c>
-      <c r="I33" s="22" t="n">
+      <c r="J33" s="22" t="n">
         <v>0.57788193</v>
       </c>
-      <c r="J33" s="23" t="n">
+      <c r="K33" s="23" t="n">
         <v>1.39</v>
       </c>
-      <c r="K33" s="22" t="n">
+      <c r="L33" s="22" t="n">
         <v>0.50739163</v>
       </c>
     </row>
@@ -12252,21 +12385,24 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G34" s="24" t="inlineStr">
+      <c r="G34" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H34" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H34" s="22" t="n">
+      <c r="I34" s="22" t="n">
         <v>1.07027397463544</v>
       </c>
-      <c r="I34" s="22" t="n">
+      <c r="J34" s="22" t="n">
         <v>0.7937623623751395</v>
       </c>
-      <c r="J34" s="23" t="n">
+      <c r="K34" s="23" t="n">
         <v>2.8800001</v>
       </c>
-      <c r="K34" s="22" t="n">
+      <c r="L34" s="22" t="n">
         <v>1.4009893</v>
       </c>
     </row>
@@ -12292,21 +12428,24 @@
       <c r="F35" s="20" t="n">
         <v/>
       </c>
-      <c r="G35" s="24" t="inlineStr">
+      <c r="G35" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H35" s="22" t="n">
+      <c r="I35" s="22" t="n">
         <v>1.068682304326143</v>
       </c>
-      <c r="I35" s="22" t="n">
+      <c r="J35" s="22" t="n">
         <v>0.6041536</v>
       </c>
-      <c r="J35" s="23" t="n">
+      <c r="K35" s="23" t="n">
         <v>1.23000005</v>
       </c>
-      <c r="K35" s="22" t="n">
+      <c r="L35" s="22" t="n">
         <v>0.45060313</v>
       </c>
     </row>
@@ -12334,23 +12473,26 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G36" s="24" t="inlineStr">
+      <c r="G36" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H36" s="22" t="n">
+      <c r="I36" s="22" t="n">
         <v>1.061212203475943</v>
       </c>
-      <c r="I36" s="22" t="n">
+      <c r="J36" s="22" t="n">
         <v>0.6916597246694085</v>
       </c>
-      <c r="J36" s="25" t="inlineStr">
+      <c r="K36" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K36" s="22" t="n">
+      <c r="L36" s="22" t="n">
         <v>0.23250532</v>
       </c>
     </row>
@@ -12376,21 +12518,24 @@
       <c r="F37" s="20" t="n">
         <v/>
       </c>
-      <c r="G37" s="21" t="inlineStr">
+      <c r="G37" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H37" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H37" s="22" t="n">
+      <c r="I37" s="22" t="n">
         <v>1.060366004632101</v>
       </c>
-      <c r="I37" s="22" t="n">
+      <c r="J37" s="22" t="n">
         <v>0.809476</v>
       </c>
-      <c r="J37" s="23" t="n">
+      <c r="K37" s="23" t="n">
         <v>4.9200002</v>
       </c>
-      <c r="K37" s="22" t="n">
+      <c r="L37" s="22" t="n">
         <v>1.9716996</v>
       </c>
     </row>
@@ -12418,21 +12563,26 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="G38" s="24" t="inlineStr">
+      <c r="G38" s="20" t="inlineStr">
+        <is>
+          <t>Chemicals</t>
+        </is>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H38" s="22" t="n">
+      <c r="I38" s="22" t="n">
         <v>1.05043788016529</v>
       </c>
-      <c r="I38" s="22" t="n">
+      <c r="J38" s="22" t="n">
         <v>0.7234581</v>
       </c>
-      <c r="J38" s="23" t="n">
+      <c r="K38" s="23" t="n">
         <v>7.27</v>
       </c>
-      <c r="K38" s="22" t="n">
+      <c r="L38" s="22" t="n">
         <v>1.872427</v>
       </c>
     </row>
@@ -12460,21 +12610,26 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G39" s="19" t="inlineStr">
+      <c r="G39" s="20" t="inlineStr">
+        <is>
+          <t>Hotels, Restaurants &amp; Leisure</t>
+        </is>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
         <is>
           <t>YELLOW</t>
         </is>
       </c>
-      <c r="H39" s="22" t="n">
+      <c r="I39" s="22" t="n">
         <v>1.048092762427114</v>
       </c>
-      <c r="I39" s="22" t="n">
+      <c r="J39" s="22" t="n">
         <v>0.65109336</v>
       </c>
-      <c r="J39" s="23" t="n">
+      <c r="K39" s="23" t="n">
         <v>9.379999999999999</v>
       </c>
-      <c r="K39" s="22" t="n">
+      <c r="L39" s="22" t="n">
         <v>0.49421084</v>
       </c>
     </row>
@@ -12502,21 +12657,26 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="G40" s="21" t="inlineStr">
+      <c r="G40" s="20" t="inlineStr">
+        <is>
+          <t>Metals &amp; Mining</t>
+        </is>
+      </c>
+      <c r="H40" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H40" s="22" t="n">
+      <c r="I40" s="22" t="n">
         <v>1.036756677485999</v>
       </c>
-      <c r="I40" s="22" t="n">
+      <c r="J40" s="22" t="n">
         <v>0.43636367</v>
       </c>
-      <c r="J40" s="23" t="n">
+      <c r="K40" s="23" t="n">
         <v>5.6500003</v>
       </c>
-      <c r="K40" s="22" t="n">
+      <c r="L40" s="22" t="n">
         <v>0.20419927</v>
       </c>
     </row>
@@ -12544,21 +12704,24 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G41" s="24" t="inlineStr">
+      <c r="G41" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H41" s="22" t="n">
+      <c r="I41" s="22" t="n">
         <v>1.030492076157528</v>
       </c>
-      <c r="I41" s="22" t="n">
+      <c r="J41" s="22" t="n">
         <v>0.4894186186926682</v>
       </c>
-      <c r="J41" s="23" t="n">
+      <c r="K41" s="23" t="n">
         <v>6.1100002</v>
       </c>
-      <c r="K41" s="22" t="n">
+      <c r="L41" s="22" t="n">
         <v>0.3481376</v>
       </c>
     </row>
@@ -12586,23 +12749,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G42" s="24" t="inlineStr">
+      <c r="G42" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H42" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H42" s="22" t="n">
+      <c r="I42" s="22" t="n">
         <v>1.028169691118431</v>
       </c>
-      <c r="I42" s="22" t="n">
+      <c r="J42" s="22" t="n">
         <v>0.7820751288732902</v>
       </c>
-      <c r="J42" s="25" t="inlineStr">
+      <c r="K42" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K42" s="22" t="n">
+      <c r="L42" s="22" t="n">
         <v>0.160262220867965</v>
       </c>
     </row>
@@ -12630,23 +12796,28 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="G43" s="24" t="inlineStr">
+      <c r="G43" s="20" t="inlineStr">
+        <is>
+          <t>Independent Power and Renewable Electricity Producers</t>
+        </is>
+      </c>
+      <c r="H43" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H43" s="22" t="n">
+      <c r="I43" s="22" t="n">
         <v>1.024547950517395</v>
       </c>
-      <c r="I43" s="22" t="n">
+      <c r="J43" s="22" t="n">
         <v>0.14083</v>
       </c>
-      <c r="J43" s="25" t="inlineStr">
+      <c r="K43" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K43" s="22" t="n">
+      <c r="L43" s="22" t="n">
         <v>0.9045904154520544</v>
       </c>
     </row>
@@ -12674,21 +12845,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G44" s="21" t="inlineStr">
+      <c r="G44" s="20" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+      <c r="H44" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H44" s="22" t="n">
+      <c r="I44" s="22" t="n">
         <v>1.021613930857689</v>
       </c>
-      <c r="I44" s="22" t="n">
+      <c r="J44" s="22" t="n">
         <v>0.8297809</v>
       </c>
-      <c r="J44" s="23" t="n">
+      <c r="K44" s="23" t="n">
         <v>5.35</v>
       </c>
-      <c r="K44" s="22" t="n">
+      <c r="L44" s="22" t="n">
         <v>0.7334186</v>
       </c>
     </row>
@@ -12716,21 +12892,24 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G45" s="24" t="inlineStr">
+      <c r="G45" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H45" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H45" s="22" t="n">
+      <c r="I45" s="22" t="n">
         <v>1.019384927967752</v>
       </c>
-      <c r="I45" s="22" t="n">
+      <c r="J45" s="22" t="n">
         <v>0.6199516180391726</v>
       </c>
-      <c r="J45" s="23" t="n">
+      <c r="K45" s="23" t="n">
         <v>4.3</v>
       </c>
-      <c r="K45" s="22" t="n">
+      <c r="L45" s="22" t="n">
         <v>2.2647114</v>
       </c>
     </row>
@@ -12758,21 +12937,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G46" s="21" t="inlineStr">
+      <c r="G46" s="20" t="inlineStr">
+        <is>
+          <t>Electrical Equipment</t>
+        </is>
+      </c>
+      <c r="H46" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H46" s="22" t="n">
+      <c r="I46" s="22" t="n">
         <v>1.019209861728622</v>
       </c>
-      <c r="I46" s="22" t="n">
+      <c r="J46" s="22" t="n">
         <v>0.41230643</v>
       </c>
-      <c r="J46" s="23" t="n">
+      <c r="K46" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="K46" s="22" t="n">
+      <c r="L46" s="22" t="n">
         <v>0.483827</v>
       </c>
     </row>
@@ -12800,23 +12984,26 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="G47" s="24" t="inlineStr">
+      <c r="G47" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H47" s="22" t="n">
+      <c r="I47" s="22" t="n">
         <v>1.015941915770137</v>
       </c>
-      <c r="I47" s="22" t="n">
+      <c r="J47" s="22" t="n">
         <v>0.183928423362757</v>
       </c>
-      <c r="J47" s="25" t="inlineStr">
+      <c r="K47" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K47" s="22" t="n">
+      <c r="L47" s="22" t="n">
         <v>0.6088967</v>
       </c>
     </row>
@@ -12844,21 +13031,26 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G48" s="21" t="inlineStr">
+      <c r="G48" s="20" t="inlineStr">
+        <is>
+          <t>Distributors</t>
+        </is>
+      </c>
+      <c r="H48" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H48" s="22" t="n">
+      <c r="I48" s="22" t="n">
         <v>1.015602077566072</v>
       </c>
-      <c r="I48" s="22" t="n">
+      <c r="J48" s="22" t="n">
         <v>0.4591028</v>
       </c>
-      <c r="J48" s="23" t="n">
+      <c r="K48" s="23" t="n">
         <v>1.72</v>
       </c>
-      <c r="K48" s="22" t="n">
+      <c r="L48" s="22" t="n">
         <v>0.5316604</v>
       </c>
     </row>
@@ -12886,21 +13078,24 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G49" s="21" t="inlineStr">
+      <c r="G49" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H49" s="21" t="inlineStr">
         <is>
           <t>GREEN</t>
         </is>
       </c>
-      <c r="H49" s="22" t="n">
+      <c r="I49" s="22" t="n">
         <v>1.012591896435186</v>
       </c>
-      <c r="I49" s="22" t="n">
+      <c r="J49" s="22" t="n">
         <v>0.4951807783269601</v>
       </c>
-      <c r="J49" s="23" t="n">
+      <c r="K49" s="23" t="n">
         <v>5.11</v>
       </c>
-      <c r="K49" s="22" t="n">
+      <c r="L49" s="22" t="n">
         <v>0.45824897</v>
       </c>
     </row>
@@ -12928,21 +13123,26 @@
           <t>Industrials</t>
         </is>
       </c>
-      <c r="G50" s="24" t="inlineStr">
+      <c r="G50" s="20" t="inlineStr">
+        <is>
+          <t>Construction &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="H50" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H50" s="22" t="n">
+      <c r="I50" s="22" t="n">
         <v>1.01079422535051</v>
       </c>
-      <c r="I50" s="22" t="n">
+      <c r="J50" s="22" t="n">
         <v>0.7220866</v>
       </c>
-      <c r="J50" s="23" t="n">
+      <c r="K50" s="23" t="n">
         <v>4.0700004</v>
       </c>
-      <c r="K50" s="22" t="n">
+      <c r="L50" s="22" t="n">
         <v>0.46383998</v>
       </c>
     </row>
@@ -12970,23 +13170,26 @@
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="G51" s="24" t="inlineStr">
+      <c r="G51" s="20" t="n">
+        <v/>
+      </c>
+      <c r="H51" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H51" s="22" t="n">
+      <c r="I51" s="22" t="n">
         <v>1.010714964634912</v>
       </c>
-      <c r="I51" s="22" t="n">
+      <c r="J51" s="22" t="n">
         <v>0.6170253471017332</v>
       </c>
-      <c r="J51" s="25" t="inlineStr">
+      <c r="K51" s="25" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="K51" s="22" t="n">
+      <c r="L51" s="22" t="n">
         <v>0.22095597</v>
       </c>
     </row>
@@ -13014,21 +13217,26 @@
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="G52" s="24" t="inlineStr">
+      <c r="G52" s="20" t="inlineStr">
+        <is>
+          <t>Textiles, Apparel &amp; Luxury Goods</t>
+        </is>
+      </c>
+      <c r="H52" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H52" s="22" t="n">
+      <c r="I52" s="22" t="n">
         <v>1.01049253958095</v>
       </c>
-      <c r="I52" s="22" t="n">
+      <c r="J52" s="22" t="n">
         <v>0.3580247</v>
       </c>
-      <c r="J52" s="23" t="n">
+      <c r="K52" s="23" t="n">
         <v>9.34</v>
       </c>
-      <c r="K52" s="22" t="n">
+      <c r="L52" s="22" t="n">
         <v>0.3563411</v>
       </c>
     </row>
@@ -13056,27 +13264,32 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="G53" s="24" t="inlineStr">
+      <c r="G53" s="20" t="inlineStr">
+        <is>
+          <t>Capital Markets</t>
+        </is>
+      </c>
+      <c r="H53" s="24" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H53" s="22" t="n">
+      <c r="I53" s="22" t="n">
         <v>1.008526545885407</v>
       </c>
-      <c r="I53" s="22" t="n">
+      <c r="J53" s="22" t="n">
         <v>0.7311028000000001</v>
       </c>
-      <c r="J53" s="23" t="n">
+      <c r="K53" s="23" t="n">
         <v>3.39</v>
       </c>
-      <c r="K53" s="22" t="n">
+      <c r="L53" s="22" t="n">
         <v>1.4634235</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
@@ -26185,10 +26398,10 @@
         <v>10</v>
       </c>
       <c r="D16" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" s="34" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate all workbooks on the audited fixes
All 23 books rebuilt (exit 0, no failures) from the corrected master:
provenance-correct EDGAR facts, single-period NNWC, reconciled forensic
ledger, DQ-gated forensic/truly scores, USD-bucketed and $2B-bounded NMS
universe, denominator-normalized tiers, haircut REIT add-back, and scores
computed after the integrity gate.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_harvard_workbook.xlsx
+++ b/asymmetry_harvard_workbook.xlsx
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -5418,7 +5418,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -6042,7 +6042,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6538,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -8022,7 +8022,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -8504,7 +8504,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -9000,7 +9000,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -10472,7 +10472,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -13939,7 +13939,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -14417,7 +14417,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -14911,7 +14911,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Mega Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -15409,7 +15409,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Large Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -15897,7 +15897,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Mega Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -16875,7 +16875,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Mega Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -19343,7 +19343,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -22287,7 +22287,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -23769,7 +23769,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Large Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>
@@ -24743,7 +24743,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
     </row>
@@ -27302,7 +27302,7 @@
       </c>
       <c r="B9" s="30" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
     </row>

</xml_diff>